<commit_message>
Revert merge of review into master (keep master unblinded)
The review branch is the anonymized copy for peer review and must not be merged
into master.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoring/ra_scoring_sheet_2.xlsx
+++ b/scoring/ra_scoring_sheet_2.xlsx
@@ -3,6 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasongeller/PreqAttention/scoring/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B13F82-78F9-7A42-B7D7-4960971354FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="37580" windowHeight="23660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>